<commit_message>
0.2.6 Provinces: Ural. Cities : Ural. (some provinces without cities due to unrealistic city names)
</commit_message>
<xml_diff>
--- a/DEFAULT_values/countries.xlsx
+++ b/DEFAULT_values/countries.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\QGIS\PROJECTS\EU4 Projet Paradoxe V2\DEFAULT_values\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B68564B3-7A6B-4E14-8B72-38EB1E36F2DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B860FD0-362F-432D-A18F-C93F9AD0A285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{49D25EAE-975A-4E0E-964A-0BF55CDC09FC}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2973" uniqueCount="2931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2976" uniqueCount="2933">
   <si>
     <t>TAG</t>
   </si>
@@ -8813,6 +8813,12 @@
   </si>
   <si>
     <t>#518D60</t>
+  </si>
+  <si>
+    <t>SWI</t>
+  </si>
+  <si>
+    <t>Swiss</t>
   </si>
 </sst>
 </file>
@@ -9654,7 +9660,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{848B17FB-53D0-4F5A-9903-753D89E7B7AA}">
-  <dimension ref="A1:F990"/>
+  <dimension ref="A1:F991"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -29457,6 +29463,26 @@
         <v>2504</v>
       </c>
     </row>
+    <row r="991" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A991" t="s">
+        <v>2931</v>
+      </c>
+      <c r="B991" t="s">
+        <v>2932</v>
+      </c>
+      <c r="C991" s="1">
+        <v>153</v>
+      </c>
+      <c r="D991" s="1">
+        <v>122</v>
+      </c>
+      <c r="E991" s="1">
+        <v>108</v>
+      </c>
+      <c r="F991" t="s">
+        <v>2730</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>